<commit_message>
Show grouped shapes and pictures on Excel sheets
Each shape or picture in a group is placed through the group's mapping of its coordinates, including nested groups.
</commit_message>
<xml_diff>
--- a/tests/corpus/xlsx/shapes.xlsx
+++ b/tests/corpus/xlsx/shapes.xlsx
@@ -344,9 +344,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
@@ -354,21 +354,71 @@
         <xdr:cNvPr id="8" name="Group"/>
         <xdr:cNvGrpSpPr/>
       </xdr:nvGrpSpPr>
-      <xdr:grpSpPr/>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2000000" cy="1000000"/>
+          <a:chOff x="1000000" y="500000"/>
+          <a:chExt cx="2000000" cy="1000000"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="9" name="Inside"/>
+          <xdr:cNvPr id="9" name="Step 1"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
+            <a:off x="1000000" y="500000"/>
+            <a:ext cx="1000000" cy="1000000"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="5B9BD5"/>
+          </a:solidFill>
         </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>Step 1</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="10" name="Step 2"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2000000" y="500000"/>
+            <a:ext cx="1000000" cy="500000"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFC000"/>
+          </a:solidFill>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>Step 2</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
       </xdr:sp>
     </xdr:grpSp>
     <xdr:clientData/>

</xml_diff>